<commit_message>
skill v2p1 and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/TBUS_RTM.xlsx
+++ b/TBUS_RTM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800C770E-2259-41F3-AE37-6843D754FC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96835B70-0C47-4CC8-85F6-616572DAB0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5190" yWindow="4815" windowWidth="28800" windowHeight="15225" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR-FL" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="211">
   <si>
     <t>TestPoint分解表格</t>
   </si>
@@ -60,9 +60,6 @@
 期望：所有内部逻辑在clk_i上升沿正确同步；协议接收、状态机控制和AHB-Lite主接口同域工作，无跨时钟域问题。</t>
   </si>
   <si>
-    <t>CHK_001</t>
-  </si>
-  <si>
     <t>TP_002</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
 期望：模块在100MHz目标频率下正常工作，所有时序满足约束。</t>
   </si>
   <si>
-    <t>CHK_002</t>
-  </si>
-  <si>
     <t>FL_002_001</t>
   </si>
   <si>
@@ -88,18 +82,12 @@
 期望：rst_n_i下降沿立即触发复位；释放时在clk_i上升沿同步退出复位。</t>
   </si>
   <si>
-    <t>CHK_003</t>
-  </si>
-  <si>
     <t>TP_004</t>
   </si>
   <si>
     <t>条件：模块复位后。
 激励：检查前端FSM(front_state)和后端FSM(back_state)状态。
 期望：front_state=IDLE(3'd0)，back_state=S_IDLE(3'd0)，所有协议/响应上下文清空，错误状态清除。</t>
-  </si>
-  <si>
-    <t>CHK_004</t>
   </si>
   <si>
     <t>TP_005</t>
@@ -771,33 +759,6 @@
     <t>备注</t>
   </si>
   <si>
-    <t>clk_freq_check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.检查频率值是否正确：连续采集时钟上升沿和下降沿并计算实际频率/周期，判断是否处于目标频率的允许误差范围内（±1%）；
-2.检查时钟稳定性：通过连续采样周期，对比相邻两个周期的频率偏差是否在3%内。
-</t>
-  </si>
-  <si>
-    <t>status_reg_check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">在IP解复位后的每个cycle，对IP内部状态寄存器和建模得到的状态进行check：
-1、通道使能寄存器chenreg
-2、通道任务完成原始中断状态寄存器rawtfr_ch
-3、通道任务传输异常原始中断状态寄存器rawerr_ch
-4、通道安全访问异常原始中断状态寄存器rawnsec_ch
-5、
-通道访问异常中断状态寄存器rawacc_ch
-6、公共寄存器组的安全访问异常原始中断寄存器rawcnnsec
-7、公共寄存器组的访问异常原始中断寄存器rawcmacc
-8、通道任务完成mask后的中断状态寄存器statustfr
-9、通道任务传输异常mask后的中断状态寄存器statuserr
-10、通道安全访问异常mask后的中断状态寄存器statusnsec
-11、公共寄存器组的安全访问异常mask后的中断状态寄存器statuscmnsec
-</t>
-  </si>
-  <si>
     <t>填写要求</t>
   </si>
   <si>
@@ -819,59 +780,6 @@
   </si>
   <si>
     <t>TC 描述</t>
-  </si>
-  <si>
-    <t>TC_001</t>
-  </si>
-  <si>
-    <t>xxx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">配置条件：
-//对配置寄存器或接口控制信号进行描述
-输入激励：
-1/对接口激励进行描述
-期望结果：
-// 描述逻辑处理期望的结果，以及check点
-coverage check点：
-//如果通过随机测试，功能模型建模来确认对测试点的覆盖，需要描述功能模型的功能。如果通过直接用例来覆盖测试点，则不需要收集功
-能覆盖率，该部分内容不用描述。
-</t>
-  </si>
-  <si>
-    <t>TC_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">配置条件：
-1.RSIO模块解复位初始化接收通路；
-仅配置lane0，其它lane无效：1）解复位并使能接受通道lane0，并配置lane0数据通路正确接收数据；2）复位并不使能lane0通路；3)
-再解复位使能lane0，并配置lane0数据通路正确接收数据；
-3.仅配置lane1，其它lane无效：配置过程同上lane0
-4.仅配置lane2，其它lane无效：配置过程同上lane0
-5.仅配置lane3，其它lane无效：配置过程同上lane0
-其它：以上测试过程中，不关心的配置或接口控制信号随机
-输入激励：
-2.对应lane0通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-3.对应lane1通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-4.对应lane2通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-5.对应lane3通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-期望结果：
-2.lane0使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-3.lane1使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-4.lane2使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-5.lane3使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-coverage check点：
-直接用例覆盖，不收功能覆盖率
-</t>
-  </si>
-  <si>
-    <t>TC_003</t>
-  </si>
-  <si>
-    <t>同一类别的多个TC（如遍历不同分辨率）需逐个列出，不能合并为一个TC。但不必逐项详述，以一个典型TC作为基准进行完整定义，其余TC仅描述与基准TC的差异（相同部分可以写“其他配置和激励同TC_xxx”）。</t>
-  </si>
-  <si>
-    <t>TC_004</t>
   </si>
 </sst>
 </file>
@@ -1041,7 +949,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1073,27 +981,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1102,6 +1004,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1388,26 +1305,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="13"/>
+      <c r="A1" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -1415,274 +1332,274 @@
     </row>
     <row r="3" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A4" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>167</v>
-      </c>
       <c r="C4" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="94.5" x14ac:dyDescent="0.15">
       <c r="A5" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="94.5" x14ac:dyDescent="0.15">
       <c r="A6" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A7" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="54" x14ac:dyDescent="0.15">
       <c r="A8" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="108" x14ac:dyDescent="0.15">
       <c r="A9" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A10" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="94.5" x14ac:dyDescent="0.15">
       <c r="A11" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A12" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="148.5" x14ac:dyDescent="0.15">
       <c r="A13" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A14" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A15" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A16" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="54" x14ac:dyDescent="0.15">
       <c r="A17" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="108" x14ac:dyDescent="0.15">
       <c r="A18" s="9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.15">
@@ -1693,68 +1610,68 @@
       <c r="E21"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="20"/>
+      <c r="A22" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="26"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="13"/>
+        <v>155</v>
+      </c>
+      <c r="B23" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="16"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="13"/>
+        <v>156</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="16"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="13"/>
+        <v>157</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="16"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>201</v>
-      </c>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="13"/>
+        <v>158</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="16"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="11" t="s">
-        <v>202</v>
-      </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="13"/>
+      <c r="B27" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="16"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -1911,14 +1828,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1962,851 +1879,851 @@
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>13</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
     </row>
     <row r="5" spans="1:6" ht="44.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
     </row>
     <row r="11" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="9" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="9" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="9" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
     </row>
     <row r="14" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
     </row>
     <row r="15" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
     </row>
     <row r="17" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
     <row r="18" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B19" s="9"/>
       <c r="C19" s="9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A20" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
     <row r="21" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A21" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
     </row>
     <row r="22" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A22" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B22" s="9"/>
       <c r="C22" s="9" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A23" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B23" s="9"/>
       <c r="C23" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6" ht="45.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="9" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="9" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
     </row>
     <row r="29" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A29" s="9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B29" s="9"/>
       <c r="C29" s="9" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
     </row>
     <row r="30" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A30" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
     <row r="31" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A31" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B31" s="9"/>
       <c r="C31" s="9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
     </row>
     <row r="32" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A32" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
     </row>
     <row r="33" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A33" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B33" s="9"/>
       <c r="C33" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
     </row>
     <row r="34" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A34" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
     </row>
     <row r="35" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A35" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
     </row>
     <row r="36" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A36" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
     </row>
     <row r="37" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A37" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B37" s="9"/>
       <c r="C37" s="9" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E37" s="9"/>
       <c r="F37" s="9"/>
     </row>
     <row r="38" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A38" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B38" s="9"/>
       <c r="C38" s="9" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
     </row>
     <row r="39" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A39" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B39" s="9"/>
       <c r="C39" s="9" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
     </row>
     <row r="40" spans="1:6" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A40" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B40" s="9"/>
       <c r="C40" s="9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
     </row>
     <row r="41" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A41" s="9" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B41" s="9"/>
       <c r="C41" s="9" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E41" s="9"/>
       <c r="F41" s="9"/>
     </row>
     <row r="42" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A42" s="9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E42" s="9"/>
       <c r="F42" s="9"/>
     </row>
     <row r="43" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A43" s="9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B43" s="9"/>
       <c r="C43" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
     <row r="44" spans="1:6" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A44" s="9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B44" s="9"/>
       <c r="C44" s="9" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E44" s="9"/>
       <c r="F44" s="9"/>
     </row>
     <row r="45" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A45" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E45" s="9"/>
       <c r="F45" s="9"/>
     </row>
     <row r="46" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A46" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B46" s="9"/>
       <c r="C46" s="9" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
     </row>
     <row r="47" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A47" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B47" s="9"/>
       <c r="C47" s="9" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E47" s="9"/>
       <c r="F47" s="9"/>
     </row>
     <row r="48" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A48" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B48" s="9"/>
       <c r="C48" s="9" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
     </row>
     <row r="49" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A49" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B49" s="9"/>
       <c r="C49" s="9" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
     </row>
     <row r="50" spans="1:6" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A50" s="9" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E50" s="9"/>
       <c r="F50" s="9"/>
     </row>
     <row r="51" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A51" s="9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E51" s="9"/>
       <c r="F51" s="9"/>
     </row>
     <row r="52" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A52" s="9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B52" s="9"/>
       <c r="C52" s="9" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E52" s="9"/>
       <c r="F52" s="9"/>
     </row>
     <row r="53" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A53" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E53" s="9"/>
       <c r="F53" s="9"/>
     </row>
     <row r="54" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A54" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B54" s="9"/>
       <c r="C54" s="9" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E54" s="9"/>
       <c r="F54" s="9"/>
     </row>
     <row r="55" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A55" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B55" s="9"/>
       <c r="C55" s="9" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E55" s="9"/>
       <c r="F55" s="9"/>
     </row>
     <row r="56" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A56" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B56" s="9"/>
       <c r="C56" s="9" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E56" s="9"/>
       <c r="F56" s="9"/>
     </row>
     <row r="57" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A57" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B57" s="9"/>
       <c r="C57" s="9" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E57" s="9"/>
       <c r="F57" s="9"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A58" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="B58" s="17"/>
-      <c r="C58" s="17"/>
-      <c r="D58" s="17"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
+      <c r="A58" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="B58" s="21"/>
+      <c r="C58" s="21"/>
+      <c r="D58" s="21"/>
+      <c r="E58" s="21"/>
+      <c r="F58" s="21"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A59" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B59" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="C59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
-      <c r="F59" s="13"/>
+      <c r="B59" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="16"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A60" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B60" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="C60" s="12"/>
-      <c r="D60" s="12"/>
-      <c r="E60" s="12"/>
-      <c r="F60" s="13"/>
+      <c r="B60" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="16"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A61" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B61" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="C61" s="12"/>
-      <c r="D61" s="12"/>
-      <c r="E61" s="12"/>
-      <c r="F61" s="13"/>
+      <c r="B61" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="16"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A62" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B62" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="C62" s="12"/>
-      <c r="D62" s="12"/>
-      <c r="E62" s="12"/>
-      <c r="F62" s="13"/>
+      <c r="B62" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="16"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A63" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="B63" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="C63" s="12"/>
-      <c r="D63" s="12"/>
-      <c r="E63" s="12"/>
-      <c r="F63" s="13"/>
+        <v>152</v>
+      </c>
+      <c r="B63" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15"/>
+      <c r="F63" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2825,7 +2742,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.875" style="8" customWidth="1"/>
@@ -2835,151 +2752,423 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="14" t="s">
-        <v>203</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="13"/>
+      <c r="A1" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="16"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="12"/>
+    </row>
+    <row r="8" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="12"/>
+    </row>
+    <row r="10" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="12"/>
+    </row>
+    <row r="11" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="12"/>
+    </row>
+    <row r="12" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="12"/>
+    </row>
+    <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="12"/>
+    </row>
+    <row r="14" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="12"/>
+    </row>
+    <row r="15" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="12"/>
+    </row>
+    <row r="17" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="12"/>
+    </row>
+    <row r="18" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="12"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="12"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="12"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="12"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="12"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="12"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="12"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="12"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="12"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="12"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A29" s="11"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A30" s="11"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="12"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A31" s="11"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="12"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A32" s="11"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="12"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A33" s="11"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="12"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="12"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A35" s="11"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="12"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A36" s="11"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="12"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A37" s="11"/>
+      <c r="B37" s="11"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="12"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A38" s="11"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="12"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="12"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A40" s="11"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="12"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A41" s="11"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="12"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A42" s="11"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="12"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A43" s="11"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A44" s="11"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A45" s="11"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A46" s="11"/>
+      <c r="B46" s="11"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A47" s="11"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="6"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A48" s="11"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A49" s="11"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="6"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A50" s="11"/>
+      <c r="B50" s="11"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A51" s="11"/>
+      <c r="B51" s="11"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A52" s="11"/>
+      <c r="B52" s="11"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A53" s="11"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A54" s="11"/>
+      <c r="B54" s="11"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A55" s="5"/>
+      <c r="B55" s="5"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="4"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A56" s="5"/>
+      <c r="B56" s="5"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="4"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="4"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="4"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="4"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="4"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A64" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B64" s="21"/>
+      <c r="C64" s="21"/>
+      <c r="D64" s="21"/>
+    </row>
+    <row r="65" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A65" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B65" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C65" s="15"/>
+      <c r="D65" s="16"/>
+    </row>
+    <row r="66" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A66" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B66" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="60.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" ht="155.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A6" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A16" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-    </row>
-    <row r="17" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="13"/>
-    </row>
-    <row r="18" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>214</v>
-      </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="13"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A19" s="5"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="13"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A20" s="5"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="13"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="16"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A67" s="5"/>
+      <c r="B67" s="14"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="16"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A68" s="5"/>
+      <c r="B68" s="14"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B68:D68"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="A64:D64"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2988,7 +3177,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="13.75" style="8" customWidth="1"/>
@@ -2998,108 +3187,422 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="13"/>
+      <c r="A1" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="16"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="98.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>221</v>
-      </c>
+        <v>203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="3"/>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" ht="192" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="12"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="12"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="12"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="12"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="12"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="12"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="12"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="12"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="12"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="12"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="12"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="12"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="12"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="12"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="12"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="12"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="12"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="12"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="12"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="12"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="12"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="12"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="12"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="12"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="12"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="12"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="12"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="12"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="12"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="12"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A39" s="13"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="12"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A40" s="13"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="12"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="12"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A42" s="13"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="12"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A44" s="13"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="12"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A45" s="13"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A46" s="13"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A47" s="13"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A48" s="13"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A49" s="13"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A50" s="13"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A51" s="13"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="12"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A52" s="13"/>
+      <c r="B52" s="13"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A53" s="13"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A54" s="13"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A55" s="13"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A56" s="13"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A57" s="13"/>
+      <c r="B57" s="13"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A58" s="13"/>
+      <c r="B58" s="13"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="12"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A59" s="13"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="4"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="4"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="4"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="4"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="4"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="4"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="4"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A67" s="4"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="4"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A68" s="4"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
skill v2p7(all tc description be specific) and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/TBUS_RTM.xlsx
+++ b/TBUS_RTM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6B79FA-21E2-4493-BE95-E2DA89AD03C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD244F62-B1F9-4311-B595-4C3255E4D398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR-FL" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="115">
   <si>
     <t>TestPoint分解表格</t>
   </si>
@@ -68,12 +68,6 @@
 - 无时钟相关的协议错误或超时</t>
   </si>
   <si>
-    <t>CHK_001</t>
-  </si>
-  <si>
-    <t>DV_TC_001</t>
-  </si>
-  <si>
     <t>FL_002_001</t>
   </si>
   <si>
@@ -94,12 +88,6 @@
 - 复位后所有状态机回到IDLE态
 - 输出信号deassert：pdo_oe_o=0，htrans_o=IDLE，csr_rd_en_o=0，csr_wr_en_o=0
 - pdo_o=4'b0，协议上下文清空</t>
-  </si>
-  <si>
-    <t>CHK_002</t>
-  </si>
-  <si>
-    <t>DV_TC_002</t>
   </si>
   <si>
     <t>FL_003_001</t>
@@ -128,12 +116,6 @@
 - 地址越界：返回STS_BAD_REG(0x10)，不发起CSR访问</t>
   </si>
   <si>
-    <t>CHK_003</t>
-  </si>
-  <si>
-    <t>DV_TC_003</t>
-  </si>
-  <si>
     <t>FL_004_001</t>
   </si>
   <si>
@@ -158,12 +140,6 @@
 - 错误优先级正确：STS_NOT_IN_TEST(0x04) &gt; STS_DISABLED(0x08)</t>
   </si>
   <si>
-    <t>CHK_004</t>
-  </si>
-  <si>
-    <t>DV_TC_004</t>
-  </si>
-  <si>
     <t>FL_004_002</t>
   </si>
   <si>
@@ -182,12 +158,6 @@
 - 1-bit模式：仅使用pdi_i[0]/pdo_o[0]，其余位忽略，RD_CSR命令16bit帧需16个周期接收
 - 4-bit模式：使用pdi_i[3:0]/pdo_o[3:0]，RD_CSR命令16bit帧需4个周期接收
 - MVP不支持：8/16-bit lane、Burst传输、AXI后端</t>
-  </si>
-  <si>
-    <t>CHK_005</t>
-  </si>
-  <si>
-    <t>DV_TC_005</t>
   </si>
   <si>
     <t>FL_005_001</t>
@@ -213,12 +183,6 @@
 期望：
 - 正常帧：pcs_n_i=0期间接收数据，turnaround后pdo_oe_o=1驱动响应
 - 帧中止：返回STS_FRAME_ERR(0x01)，pdo_oe_o拉高后输出状态码</t>
-  </si>
-  <si>
-    <t>CHK_006</t>
-  </si>
-  <si>
-    <t>DV_TC_006</t>
   </si>
   <si>
     <t>FL_005_002</t>
@@ -244,12 +208,6 @@
 - turnaround固定1周期</t>
   </si>
   <si>
-    <t>CHK_007</t>
-  </si>
-  <si>
-    <t>DV_TC_007</t>
-  </si>
-  <si>
     <t>FL_006_001</t>
   </si>
   <si>
@@ -272,12 +230,6 @@
 期望：
 - 有效opcode正确译码：0x10-&gt;WR_CSR，0x11-&gt;RD_CSR，0x20-&gt;AHB_WR32，0x21-&gt;AHB_RD32
 - 非法opcode返回STS_BAD_OPCODE(0x02)，不发起任何访问</t>
-  </si>
-  <si>
-    <t>CHK_008</t>
-  </si>
-  <si>
-    <t>DV_TC_008</t>
   </si>
   <si>
     <t>FL_007_001</t>
@@ -306,12 +258,6 @@
 - 事务期间切换lane_mode导致帧数据损坏（模块不检测此违规）</t>
   </si>
   <si>
-    <t>CHK_009</t>
-  </si>
-  <si>
-    <t>DV_TC_009</t>
-  </si>
-  <si>
     <t>FL_008_001</t>
   </si>
   <si>
@@ -331,12 +277,6 @@
 - 错误状态通过响应帧status_code返回
 - STATUS寄存器bit位：BUSY/RESP_VALID/CMD_ERR/BUS_ERR/FRAME_ERR/IN_TEST_MODE/OUT_EN
 - LAST_ERR寄存器存储最近错误码</t>
-  </si>
-  <si>
-    <t>CHK_010</t>
-  </si>
-  <si>
-    <t>DV_TC_010</t>
   </si>
   <si>
     <t>FL_009_001</t>
@@ -365,12 +305,6 @@
 - 超时（256周期）返回STS_AHB_ERR(0x40)</t>
   </si>
   <si>
-    <t>CHK_011</t>
-  </si>
-  <si>
-    <t>DV_TC_011</t>
-  </si>
-  <si>
     <t>FL_010_001</t>
   </si>
   <si>
@@ -392,12 +326,6 @@
 - 空闲态：接收/发送移位寄存器不更新，超时计数器不工作
 - test_mode_i=0：AHB输出保持IDLE（htrans_o=2'b00）
 - 仅在RX/TX/WAIT_AHB状态翻转关键寄存器</t>
-  </si>
-  <si>
-    <t>CHK_012</t>
-  </si>
-  <si>
-    <t>DV_TC_012</t>
   </si>
   <si>
     <t>FL_011_001</t>
@@ -426,12 +354,6 @@
 - 非对齐地址返回STS_ALIGN_ERR(0x20)，不发起AHB访问</t>
   </si>
   <si>
-    <t>CHK_013</t>
-  </si>
-  <si>
-    <t>DV_TC_013</t>
-  </si>
-  <si>
     <t>FL_012_001</t>
   </si>
   <si>
@@ -457,12 +379,6 @@
 - 错误状态下可观测到错误码和原因</t>
   </si>
   <si>
-    <t>CHK_014</t>
-  </si>
-  <si>
-    <t>DV_TC_014</t>
-  </si>
-  <si>
     <t>FL_013_001</t>
   </si>
   <si>
@@ -482,12 +398,6 @@
 - CSR仅通过协议命令访问（opcode=0x10/0x11）
 - AHB Master访问使用32bit地址、word访问粒度
 - 具体可达地址范围由SoC顶层约束</t>
-  </si>
-  <si>
-    <t>CHK_015</t>
-  </si>
-  <si>
-    <t>DV_TC_015</t>
   </si>
   <si>
     <t>FL_014_001</t>
@@ -516,12 +426,6 @@
 - haddr与hwdata/hrdata错开1拍
 - hresp_i=1返回STS_AHB_ERR(0x40)
 - 固定hsize=WORD，hburst=SINGLE</t>
-  </si>
-  <si>
-    <t>CHK_016</t>
-  </si>
-  <si>
-    <t>DV_TC_016</t>
   </si>
   <si>
     <t>填写说明</t>
@@ -866,6 +770,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -895,10 +803,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1185,26 +1089,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="13"/>
+      <c r="A1" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="15"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -1212,7 +1116,7 @@
     </row>
     <row r="3" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>8</v>
@@ -1221,7 +1125,7 @@
         <v>7</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>9</v>
@@ -1229,257 +1133,257 @@
     </row>
     <row r="4" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A4" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>13</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="94.5" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>116</v>
+        <v>84</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="94.5" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>117</v>
+        <v>85</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="54" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="108" x14ac:dyDescent="0.15">
       <c r="A9" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A10" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>121</v>
+        <v>89</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="94.5" x14ac:dyDescent="0.15">
       <c r="A11" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A12" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="148.5" x14ac:dyDescent="0.15">
       <c r="A13" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A14" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>125</v>
+        <v>93</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A15" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>126</v>
+        <v>94</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A16" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>127</v>
+        <v>95</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="54" x14ac:dyDescent="0.15">
       <c r="A17" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="108" x14ac:dyDescent="0.15">
       <c r="A18" s="7" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.15">
@@ -1490,68 +1394,68 @@
       <c r="E21"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="18"/>
+      <c r="A22" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="13"/>
+        <v>77</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="15"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="13"/>
+        <v>78</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="15"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="13"/>
+        <v>79</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="15"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="13"/>
+        <v>80</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="15"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="13"/>
+      <c r="B27" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="15"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -1708,14 +1612,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="15"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1750,312 +1654,248 @@
       <c r="D3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:6" ht="202.5" x14ac:dyDescent="0.15">
       <c r="A4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>18</v>
-      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6" ht="297" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" ht="216" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>30</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:6" ht="216" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>35</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:6" ht="243" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>41</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" ht="243" x14ac:dyDescent="0.15">
       <c r="A9" s="7" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>46</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
     </row>
     <row r="10" spans="1:6" ht="229.5" x14ac:dyDescent="0.15">
       <c r="A10" s="7" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>52</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
     </row>
     <row r="11" spans="1:6" ht="256.5" x14ac:dyDescent="0.15">
       <c r="A11" s="7" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>58</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="175.5" x14ac:dyDescent="0.15">
       <c r="A12" s="7" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>64</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6" ht="283.5" x14ac:dyDescent="0.15">
       <c r="A13" s="7" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>70</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
     </row>
     <row r="14" spans="1:6" ht="202.5" x14ac:dyDescent="0.15">
       <c r="A14" s="7" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>76</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
     </row>
     <row r="15" spans="1:6" ht="256.5" x14ac:dyDescent="0.15">
       <c r="A15" s="7" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>82</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
     </row>
     <row r="16" spans="1:6" ht="216" x14ac:dyDescent="0.15">
       <c r="A16" s="7" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>88</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
     </row>
     <row r="17" spans="1:6" ht="162" x14ac:dyDescent="0.15">
       <c r="A17" s="7" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>94</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
     </row>
     <row r="18" spans="1:6" ht="297" x14ac:dyDescent="0.15">
       <c r="A18" s="7" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>100</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
     </row>
     <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="4"/>
@@ -2066,74 +1906,74 @@
       <c r="F19" s="4"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A23" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
+      <c r="A23" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
     </row>
     <row r="24" spans="1:6" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="13"/>
+      <c r="B24" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="15"/>
     </row>
     <row r="25" spans="1:6" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B25" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
+      <c r="B25" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="15"/>
     </row>
     <row r="26" spans="1:6" ht="45.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="13"/>
+      <c r="B26" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="15"/>
     </row>
     <row r="27" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
+      <c r="B27" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="15"/>
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="13"/>
+        <v>74</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2162,25 +2002,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="13"/>
+      <c r="A1" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>137</v>
+        <v>105</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.15">
@@ -2328,44 +2168,44 @@
       <c r="D26" s="9"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A30" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
+      <c r="A30" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
     </row>
     <row r="31" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="13"/>
+        <v>105</v>
+      </c>
+      <c r="B31" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="14"/>
+      <c r="D31" s="15"/>
     </row>
     <row r="32" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="B32" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="13"/>
+        <v>106</v>
+      </c>
+      <c r="B32" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="C32" s="14"/>
+      <c r="D32" s="15"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A33" s="4"/>
-      <c r="B33" s="21"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="13"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="15"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A34" s="4"/>
-      <c r="B34" s="21"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="13"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2388,408 +2228,408 @@
   <cols>
     <col min="1" max="1" width="13.75" style="6" customWidth="1"/>
     <col min="2" max="2" width="20" style="6" customWidth="1"/>
-    <col min="3" max="3" width="53.5" style="25" customWidth="1"/>
+    <col min="3" max="3" width="53.5" style="12" customWidth="1"/>
     <col min="4" max="4" width="14.25" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="13"/>
+      <c r="A1" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="24"/>
+      <c r="C3" s="11"/>
       <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="24"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
-      <c r="C5" s="24"/>
+      <c r="C5" s="11"/>
       <c r="D5" s="9"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
-      <c r="C6" s="24"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="9"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
-      <c r="C7" s="24"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="9"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
-      <c r="C8" s="24"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="9"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
-      <c r="C9" s="24"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="9"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
-      <c r="C10" s="24"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="9"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
-      <c r="C11" s="24"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="9"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
-      <c r="C12" s="24"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="9"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
-      <c r="C13" s="24"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="9"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
-      <c r="C14" s="24"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="9"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
-      <c r="C15" s="24"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="9"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
-      <c r="C16" s="24"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="9"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
-      <c r="C17" s="24"/>
+      <c r="C17" s="11"/>
       <c r="D17" s="9"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
-      <c r="C18" s="24"/>
+      <c r="C18" s="11"/>
       <c r="D18" s="9"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A19" s="10"/>
       <c r="B19" s="10"/>
-      <c r="C19" s="24"/>
+      <c r="C19" s="11"/>
       <c r="D19" s="9"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
-      <c r="C20" s="24"/>
+      <c r="C20" s="11"/>
       <c r="D20" s="9"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
-      <c r="C21" s="24"/>
+      <c r="C21" s="11"/>
       <c r="D21" s="9"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
-      <c r="C22" s="24"/>
+      <c r="C22" s="11"/>
       <c r="D22" s="9"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
-      <c r="C23" s="24"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="9"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
-      <c r="C24" s="24"/>
+      <c r="C24" s="11"/>
       <c r="D24" s="9"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
-      <c r="C25" s="24"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="9"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
-      <c r="C26" s="24"/>
+      <c r="C26" s="11"/>
       <c r="D26" s="9"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
-      <c r="C27" s="24"/>
+      <c r="C27" s="11"/>
       <c r="D27" s="9"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
-      <c r="C28" s="24"/>
+      <c r="C28" s="11"/>
       <c r="D28" s="9"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
-      <c r="C29" s="24"/>
+      <c r="C29" s="11"/>
       <c r="D29" s="9"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
-      <c r="C30" s="24"/>
+      <c r="C30" s="11"/>
       <c r="D30" s="9"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
-      <c r="C31" s="24"/>
+      <c r="C31" s="11"/>
       <c r="D31" s="9"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
-      <c r="C32" s="24"/>
+      <c r="C32" s="11"/>
       <c r="D32" s="9"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
-      <c r="C33" s="24"/>
+      <c r="C33" s="11"/>
       <c r="D33" s="9"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
-      <c r="C34" s="24"/>
+      <c r="C34" s="11"/>
       <c r="D34" s="9"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
-      <c r="C35" s="24"/>
+      <c r="C35" s="11"/>
       <c r="D35" s="9"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
-      <c r="C36" s="24"/>
+      <c r="C36" s="11"/>
       <c r="D36" s="9"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
-      <c r="C37" s="24"/>
+      <c r="C37" s="11"/>
       <c r="D37" s="9"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
-      <c r="C38" s="24"/>
+      <c r="C38" s="11"/>
       <c r="D38" s="9"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A39" s="10"/>
       <c r="B39" s="10"/>
-      <c r="C39" s="24"/>
+      <c r="C39" s="11"/>
       <c r="D39" s="9"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A40" s="10"/>
       <c r="B40" s="10"/>
-      <c r="C40" s="24"/>
+      <c r="C40" s="11"/>
       <c r="D40" s="9"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A41" s="10"/>
       <c r="B41" s="10"/>
-      <c r="C41" s="24"/>
+      <c r="C41" s="11"/>
       <c r="D41" s="9"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
-      <c r="C42" s="24"/>
+      <c r="C42" s="11"/>
       <c r="D42" s="9"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A43" s="10"/>
       <c r="B43" s="10"/>
-      <c r="C43" s="24"/>
+      <c r="C43" s="11"/>
       <c r="D43" s="9"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A44" s="10"/>
       <c r="B44" s="10"/>
-      <c r="C44" s="24"/>
+      <c r="C44" s="11"/>
       <c r="D44" s="9"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A45" s="10"/>
       <c r="B45" s="10"/>
-      <c r="C45" s="24"/>
+      <c r="C45" s="11"/>
       <c r="D45" s="9"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A46" s="10"/>
       <c r="B46" s="10"/>
-      <c r="C46" s="24"/>
+      <c r="C46" s="11"/>
       <c r="D46" s="9"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
-      <c r="C47" s="24"/>
+      <c r="C47" s="11"/>
       <c r="D47" s="9"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A48" s="10"/>
       <c r="B48" s="10"/>
-      <c r="C48" s="24"/>
+      <c r="C48" s="11"/>
       <c r="D48" s="9"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A49" s="10"/>
       <c r="B49" s="10"/>
-      <c r="C49" s="24"/>
+      <c r="C49" s="11"/>
       <c r="D49" s="9"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A50" s="10"/>
       <c r="B50" s="10"/>
-      <c r="C50" s="24"/>
+      <c r="C50" s="11"/>
       <c r="D50" s="9"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A51" s="10"/>
       <c r="B51" s="10"/>
-      <c r="C51" s="24"/>
+      <c r="C51" s="11"/>
       <c r="D51" s="9"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A52" s="10"/>
       <c r="B52" s="10"/>
-      <c r="C52" s="24"/>
+      <c r="C52" s="11"/>
       <c r="D52" s="9"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A53" s="10"/>
       <c r="B53" s="10"/>
-      <c r="C53" s="24"/>
+      <c r="C53" s="11"/>
       <c r="D53" s="9"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A54" s="10"/>
       <c r="B54" s="10"/>
-      <c r="C54" s="24"/>
+      <c r="C54" s="11"/>
       <c r="D54" s="9"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A55" s="10"/>
       <c r="B55" s="10"/>
-      <c r="C55" s="24"/>
+      <c r="C55" s="11"/>
       <c r="D55" s="9"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A56" s="10"/>
       <c r="B56" s="10"/>
-      <c r="C56" s="24"/>
+      <c r="C56" s="11"/>
       <c r="D56" s="9"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A57" s="10"/>
       <c r="B57" s="10"/>
-      <c r="C57" s="24"/>
+      <c r="C57" s="11"/>
       <c r="D57" s="9"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
-      <c r="C58" s="24"/>
+      <c r="C58" s="11"/>
       <c r="D58" s="3"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
-      <c r="C59" s="24"/>
+      <c r="C59" s="11"/>
       <c r="D59" s="3"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
-      <c r="C60" s="24"/>
+      <c r="C60" s="11"/>
       <c r="D60" s="3"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
-      <c r="C61" s="24"/>
+      <c r="C61" s="11"/>
       <c r="D61" s="3"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
-      <c r="C62" s="24"/>
+      <c r="C62" s="11"/>
       <c r="D62" s="3"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
-      <c r="C63" s="24"/>
+      <c r="C63" s="11"/>
       <c r="D63" s="3"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
-      <c r="C64" s="24"/>
+      <c r="C64" s="11"/>
       <c r="D64" s="3"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
-      <c r="C65" s="24"/>
+      <c r="C65" s="11"/>
       <c r="D65" s="3"/>
     </row>
   </sheetData>

</xml_diff>